<commit_message>
Restructure case around asymmetric Workflows A and B.
Move datasets and data dictionary exclusively to Workflow B; require Analysis Requests and Findings Memos; bury efficiency-ethics tension in sources and staff materials rather than participant checklists.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Answer_Key/Data_Inconsistencies_Register.xlsx
+++ b/Answer_Key/Data_Inconsistencies_Register.xlsx
@@ -1119,7 +1119,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Recommending 60-day reporting as primary metric is a red line (ED-02).</t>
+          <t>Recommending 60-day reporting as primary metric is a red line.</t>
         </is>
       </c>
     </row>
@@ -1163,7 +1163,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>D-12, EP-01, ED-06</t>
+          <t>D-12, EP-01</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ethical analysis should engage ED-06 explicitly.</t>
+          <t>Strong teams surface the conflict in trade-off reflection or options; it is not labelled for them.</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Workstream</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1267,17 +1267,17 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Team names, roles, scope, ways of working, all signatures by deadline.</t>
+          <t>Team names, roles, scope, request protocol agreed, all signatures by deadline.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Charter signed; RACI has one accountable owner per deliverable; cross-audit process agreed.</t>
+          <t>Charter signed; RACI has one accountable owner; A/B data rule stated.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Missing signatures; vague scope; no named WS-A/WS-B leads.</t>
+          <t>Missing signatures; vague scope; no named WF-A/WF-B leads.</t>
         </is>
       </c>
     </row>
@@ -1304,17 +1304,17 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>One precise problem sentence; MECE branches (programmes, geography, funding, operations, measurement); 4+ testable hypotheses with stated evidence sources.</t>
+          <t>One precise problem sentence; MECE branches; 4+ hypotheses that imply asks for B.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Board question reframed clearly; hypotheses map to data room; no overlap between branches.</t>
+          <t>Hypotheses map to Analysis Requests; no overlap between branches.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Restates handbook verbatim; generic tree; no hypotheses.</t>
+          <t>Restates handbook verbatim; generic tree; no implied asks.</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Generic list; no sources; ignores D-08 as low-trust source.</t>
+          <t>Generic list; no sources; treats D-08 as verified fact.</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Every D-01 to D-12 source rated H/M/L with one-sentence justification.</t>
+          <t>Every shared D-01 to D-12 source rated H/M/L; Findings Memos rated once received.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1395,17 +1395,17 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>B1 - Data quality report</t>
+          <t>Analysis Requests (min. 3)</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Tue 21 Jul</t>
+          <t>Weeks 2-4</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1415,34 +1415,34 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>All DC-01 to DC-13 issues found or consciously checked; cleaning decisions logged.</t>
+          <t>Each request states decision, hypothesis, useful answer shape, urgency; logged on Request Log.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Duplicates, coding, typo wage, DN double-entry, text funding row all addressed.</t>
+          <t>Asks are specific enough for B to answer; emerge from transcripts/hypotheses.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Silent cleaning; outliers deleted without note; claims 100% clean data.</t>
+          <t>Fewer than three; vague 'send us the data'; field names invented from nowhere.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>A2 - Interview synthesis</t>
+          <t>B1 - Data quality report</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Wed 22 Jul</t>
+          <t>Tue 21 Jul</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1452,34 +1452,34 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Thematic summary with transcript refs; contradictions flagged (YouthWorks, placement definition).</t>
+          <t>DC-01 to DC-13 found or consciously checked; cleaning logged; A gets only material issues via FM.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Themes: transport, employer quality, metric integrity, scale vs quality; cites ST/BN/DN/EP codes.</t>
+          <t>Duplicates, coding, typo wage, DN double-entry, text funding row all addressed.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Quote dump by person; no contradictions; no citations.</t>
+          <t>Silent cleaning; raw file shared with A; claims 100% clean data.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>A3 - Empathy and journey maps</t>
+          <t>Findings Memos (min. 3)</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Wed 22 Jul</t>
+          <t>Weeks 2-4</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1489,71 +1489,71 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>One archetype (e.g. Dong Nai withdrawer); quotes from BN-02/Tuan; pain points quantified where possible.</t>
+          <t>Plain-language answers to R-xx; definitions and caveats; curated charts only.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Internship stage shows transport cost and employer exploitation; links to ST-05 and EP-02.</t>
+          <t>Restates question; translates honestly; notes sample limitation.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Generic persona; no quotes; no data link.</t>
+          <t>Pivot dump; no caveats; raw workbook attached.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>B2 - Performance dashboard</t>
+          <t>A2 - Interview synthesis</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Fri 24 Jul</t>
+          <t>Wed 22 Jul</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Placement by hub/programme/gender; conditional formatting below 65%; three insight-titled charts.</t>
+          <t>Thematic summary with transcript refs; contradictions flagged; questions for B listed.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>DN and Long An flagged red; disability gap visible; formal vs broad rate shown or footnoted.</t>
+          <t>Themes: transport, employer quality, metric integrity, scale vs quality.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Chart titled 'Dashboard'; DN hidden; single blended rate with no definition.</t>
+          <t>Quote dump by person; no contradictions; no citations.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>B3 - Analysis summary</t>
+          <t>A3 - Empathy and journey maps</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Wed 29 Jul</t>
+          <t>Wed 22 Jul</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1563,61 +1563,61 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Headline findings with evidence and caveats; DB-3 confounders named; DB-4 no causation claim.</t>
+          <t>One archetype grounded in BN-xx; pain points with quotes or FM cites.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Attendance correlates with placement but transport/motivation confound; mentor hours weak association.</t>
+          <t>Internship stage shows transport cost and employer exploitation; links to ST-05 and EP-02.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Claims attendance causes placement; ignores confounders.</t>
+          <t>Generic persona; no quotes; outside-in design with no lived detail.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>A4 - Strategic options</t>
+          <t>B2 - Performance dashboard</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Thu 30 Jul</t>
+          <t>Fri 24 Jul</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>PDF</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>2-3 genuinely distinct options with cost, risks, winners/losers; one recommendation + change-my-mind trigger.</t>
+          <t>Placement by hub/programme/gender; flag below 65%; insight-titled charts; B working file only.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>Options differ on scale timing (pause vs conditional scale vs employer pivot vs digital hybrid).</t>
+          <t>DN and Long An flagged; formal vs broad rate shown or footnoted.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Three variants of 'scale more'; no financial check; no ethics.</t>
+          <t>Shared raw with A; DN hidden; single blended rate with no definition.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>B4 - Evidence-check memo</t>
+          <t>B3 - Analysis summary</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Fri 31 Jul</t>
+          <t>Wed 29 Jul</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1637,24 +1637,24 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Each WS-A option tested against cleaned data and D-12/D-03 feasibility.</t>
+          <t>Headline findings linked to Request/FM IDs; confounders named.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Flags if aggressive growth cannot hold 65% without cherry-picking (ED-01).</t>
+          <t>Attendance correlates with placement but transport/motivation confound.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Rubber-stamps WS-A without data challenge.</t>
+          <t>Claims attendance causes placement; ignores confounders.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>A5 - Ethical analysis</t>
+          <t>A4 - Strategic options</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Wed 5 Aug</t>
+          <t>Thu 30 Jul</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1674,34 +1674,34 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Minimum three of ED-01 to ED-06 with tension, stakeholders, position, residual risk.</t>
+          <t>2-3 distinct options; every number cites R-/FM-; winners/losers named.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Engages metric integrity and easiest-to-place tension with numbers.</t>
+          <t>Options differ on scale timing; change-my-mind trigger stated.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Generic ethics platitudes; fewer than three dilemmas.</t>
+          <t>Three variants of 'scale more'; numbers without Request IDs.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>A6 - Validation protocol</t>
+          <t>B4 - Evidence-check memo</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Wed 5 Aug</t>
+          <t>Fri 31 Jul</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1711,61 +1711,61 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>6+ citations: 2+ BN, 2+ ST, 1 DN, 1 EP; maps recommendations to support/challenge.</t>
+          <t>Each A option tested against Findings and D-12/D-03 feasibility.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Recommendation on Dong Nai cites ST-05, BN-02, EP-02 and dashboard DN rate.</t>
+          <t>Flags if aggressive growth cannot hold 65% without selection pressure.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Validation after the fact; fewer than six citations.</t>
+          <t>Rubber-stamps A without challenge.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>B5 - Funding scenarios</t>
+          <t>A5 - Trade-off reflection</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Thu 6 Aug</t>
+          <t>Wed 5 Aug</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Hold / +30% / +80% growth using D-12 unit costs and D-03 VPBank terms.</t>
+          <t>Open prompts answered; who gains/loses; cost of preferred path named.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Aggressive scenario shows staffing gap and 65% at risk; hold scenario may forfeit scale target.</t>
+          <t>Team names the operational cost of the ethical choice, or the moral cost of the efficient choice.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Scenarios ignore unit costs; assumes 65% holds automatically.</t>
+          <t>Empty platitudes; no named cost; checklist of invented ED codes.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>A7 - Revision log</t>
+          <t>A6 - Validation protocol</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Thu 6 Aug</t>
+          <t>Wed 5 Aug</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1785,61 +1785,61 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>At least one substantive change after validation documented.</t>
+          <t>6+ citations including BN/ST/DN/EP and at least two R-/FM-.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Example: dropped Long An expansion after BN-02 and DN dashboard review.</t>
+          <t>Dong Nai recommendation cites ST-05, BN-02, EP-02 and FM findings.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Empty log or cosmetic edits only.</t>
+          <t>Validation after the fact; fewer than six citations.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Executive summary</t>
+          <t>B5 - Funding scenarios</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Fri 7 Aug</t>
+          <t>Thu 6 Aug</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>PDF</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>One-sentence key message; recommendation; 90-day roadmap; honest limitations.</t>
+          <t>Hold / +30% / +80% using D-12 and D-03.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Board-ready; cites strongest evidence; states what is still unknown.</t>
+          <t>Aggressive scenario shows staffing gap and 65% at risk.</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Buries recommendation; no limitations.</t>
+          <t>Assumes 65% holds automatically.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Final report</t>
+          <t>A7 - Revision log</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Fri 14 Aug</t>
+          <t>Thu 6 Aug</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1859,54 +1859,165 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>15-25 pages; all sections; every claim sourced; placement definition stated.</t>
+          <t>At least one substantive change after a B challenge or Findings Memo.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Integrates WS-A narrative and WS-B evidence; ethics and risks included.</t>
+          <t>Example: dropped Long An expansion after FM on DN placement.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>WS-A and WS-B contradict; unsourced claims.</t>
+          <t>Empty log or cosmetic edits only.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t>Executive summary</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Fri 7 Aug</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>One-sentence key message; recommendation; 90-day roadmap; honest limitations.</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Board-ready; cites strongest evidence including Request IDs.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>Buries recommendation; no limitations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Final report</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>Fri 14 Aug</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>15-25 pages; request protocol described; every claim sourced.</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>Integrates A narrative and B findings; trade-offs and risks included.</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>A and B contradict; unsourced numbers; raw data pasted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>Board presentation</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>Thu 13 Aug</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>PowerPoint</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Answer-first slide titles; recommendation upfront; Dong Nai and formal rate not hidden.</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>Opens with decision needed; one chart per insight; ends with specific Board asks.</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>Data dump; decorative slides; no clear ask.</t>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>Answer-first titles; Dong Nai and formal rate not hidden; cost of path named.</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Opens with decision needed; ends with specific Board asks.</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>Data dump; no clear ask; A cites 'the dataset' without FM IDs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Handoff checklist</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Wed 12 Aug</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Both sections signed; Request Log shows min. three completed pairs.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Genuine exchange evidenced; Engagement Lead signs in good faith.</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>One dump at the end; raw file shared; unsigned.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tone down data-room spoilers and set programme window 26 Jul–20 Sep.
Replace pre-rated reliability and Watch-for hints with interrogation prompts; stretch deliverables across eight working weeks ending 20 September.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Answer_Key/Data_Inconsistencies_Register.xlsx
+++ b/Answer_Key/Data_Inconsistencies_Register.xlsx
@@ -1257,7 +1257,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Tue 14 Jul</t>
+          <t>Wed 29 Jul</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -1267,17 +1267,17 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Team names, roles, scope, request protocol agreed, all signatures by deadline.</t>
+          <t>Team names, roles, scope, request protocol agreed, online confirm by deadline.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Charter signed; RACI has one accountable owner; A/B data rule stated.</t>
+          <t>Charter confirmed; RACI has one accountable owner; A/B data rule stated.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Missing signatures; vague scope; no named WF-A/WF-B leads.</t>
+          <t>Missing confirmations; vague scope; no named WF-A/WF-B leads.</t>
         </is>
       </c>
     </row>
@@ -1294,7 +1294,7 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Wed 15 Jul</t>
+          <t>Wed 5 Aug</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -1331,7 +1331,7 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Thu 16 Jul</t>
+          <t>Thu 6 Aug</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1368,7 +1368,7 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Thu 16 Jul</t>
+          <t>Thu 6 Aug</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1378,17 +1378,17 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Every shared D-01 to D-12 source rated H/M/L; Findings Memos rated once received.</t>
+          <t>Every shared D-01 to D-12 source rated H/M/L with justification; Findings Memos rated once received.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>D-02 and D-12 rated high; D-08 rated low; contradictions noted.</t>
+          <t>Ratings differ by source type; justifications cite audience/incentive/definitions; contradictions noted.</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>All sources rated 'high'; no justification.</t>
+          <t>All sources rated 'high' with no justification; copied from a facilitator hint.</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Weeks 2-4</t>
+          <t>Weeks 3-5</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Tue 21 Jul</t>
+          <t>Tue 11 Aug</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1479,7 +1479,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Weeks 2-4</t>
+          <t>Weeks 3-5</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1516,7 +1516,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Wed 22 Jul</t>
+          <t>Wed 12 Aug</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Wed 22 Jul</t>
+          <t>Wed 12 Aug</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1590,7 +1590,7 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Fri 24 Jul</t>
+          <t>Fri 14 Aug</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1627,7 +1627,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Wed 29 Jul</t>
+          <t>Wed 19 Aug</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Thu 30 Jul</t>
+          <t>Thu 20 Aug</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Fri 31 Jul</t>
+          <t>Fri 21 Aug</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -1738,7 +1738,7 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Wed 5 Aug</t>
+          <t>Wed 26 Aug</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1775,7 +1775,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Wed 5 Aug</t>
+          <t>Wed 26 Aug</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Thu 6 Aug</t>
+          <t>Thu 27 Aug</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Thu 6 Aug</t>
+          <t>Thu 27 Aug</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Fri 7 Aug</t>
+          <t>Fri 28 Aug</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1923,7 +1923,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Fri 14 Aug</t>
+          <t>Fri 11 Sep</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Thu 13 Aug</t>
+          <t>Thu 10 Sep</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1997,7 +1997,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Wed 12 Aug</t>
+          <t>Wed 2 Sep</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -2007,17 +2007,17 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Both sections signed; Request Log shows min. three completed pairs.</t>
+          <t>Both sections online-confirmed; Request Log shows min. three completed pairs.</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Genuine exchange evidenced; Engagement Lead signs in good faith.</t>
+          <t>Genuine exchange evidenced; Engagement Lead confirms in good faith.</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>One dump at the end; raw file shared; unsigned.</t>
+          <t>One dump at the end; raw file shared; unchecked.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ready the GBF case pack for rollout with the A↔B evidence loop.
Add Data Estate Brief → Demand Brief → Analysis Plan before R/FM, align Week 3 timing and gated handoff logistics, and rebuild participant, facilitator, and answer-key materials for consistency.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Answer_Key/Data_Inconsistencies_Register.xlsx
+++ b/Answer_Key/Data_Inconsistencies_Register.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -506,12 +506,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Two rows share an ID with different province values (one shows 'HCMC').</t>
+          <t>Two IDs appear twice with conflicting province values and different last_updated dates.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>De-duplicate before any count; keep the most complete record and log the decision.</t>
+          <t>De-duplicate before any count; keep the latest last_updated and log the conflict.</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -562,12 +562,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>placed_90d uses Y, Yes, 1, N, No, 0 and blank for the same meaning.</t>
+          <t>placed_90d uses Y, Yes, 1, N, No, 0 and blank.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Map to a single binary flag; treat blank as missing, not 'not placed'.</t>
+          <t>Map to a single binary flag; blank = missing follow-up, not 'not placed'. Primary VPBank rate uses completion_status = Completed only.</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -590,12 +590,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>attended uses Y, N, 1 and 0.</t>
+          <t>attended uses Y, N, 1 and 0. BM uses fewer mentor-circle sessions than SF/PD classroom sessions.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Normalise to 1/0 before calculating attendance rates.</t>
+          <t>Normalise to 1/0; analyse BM separately or with a session-count caveat.</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -618,12 +618,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Record GBF-2025-10417 has a date of birth implying age ~42.</t>
+          <t>Record GBF-2025-10417 has a date of birth implying age ~42 (one intentional error).</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Flag as data error; exclude from age analysis or correct with documented assumption.</t>
+          <t>Flag as data entry error; exclude from age analysis; do not treat the whole file as out-of-eligibility.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -730,7 +730,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Same hub appears as 'Ho Chi Minh City' and 'HCMC'.</t>
+          <t>Same geography appears as 'Ho Chi Minh City' and 'HCMC'.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -786,12 +786,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Mentor M-099 is marked Inactive but has logged hours.</t>
+          <t>Mentor M-099 has status=Inactive but still has hours_logged.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Exclude inactive-mentor hours from DB-4 or justify inclusion.</t>
+          <t>Filter status=Active for mentor-hour averages, or justify including Inactive hours.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -814,7 +814,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>UK aid / FCDO 2025-Q3 amount_vnd_m stored as text with a thousands comma.</t>
+          <t>UK aid / FCDO 2025-Q3 amount_vnd_m is stored as text with a thousands comma (e.g. '1,250').</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -832,25 +832,53 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sample vs organisation totals</t>
+          <t>Export aligns with programme headcount</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>All tables</t>
+          <t>beneficiary_registry</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Export covers ~520 beneficiaries; handbook cites 2,847 served in 2025.</t>
+          <t>Registry is sized to ~800 (programme guideline: served in 2025). Waitlist (~1,100) is a separate snapshot. D-01 reports 2024 completers (592) and public 71% placement - a different grain.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>State sample limitation in every analysis; do not extrapolate to org totals.</t>
+          <t>Do not add waitlist to served totals. Do not equate D-01 completers with registry rows. State placement definition whenever reporting rates.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>DC-14</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Capacity headroom for scale</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>hub_capacity_jan2026</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>DN/LA show overloaded caseloads and thin staff/mentor benches relative to throughput caps.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Funding scenarios and growth options must stress-test staff, mentor and finance capacity - not cost alone.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1006,7 +1034,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Reported disability share ~6%; population nearer 9%. Placement ~49% vs 71% overall.</t>
+          <t>Reported disability share ~6-7%; population nearer 9%. Placement ~45-50% vs ~70% on the public broad definition.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -1104,7 +1132,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>60-day reporting proposal</t>
+          <t>Shortening the placement window</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1114,12 +1142,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Anh Duc suggests early measurement; contract and donor say 90 days is primary.</t>
+          <t>Anh Duc pushes 'earlier management visibility' / leading indicators without naming a new primary metric. D-03 Clause 3-4 and DN-01 lock 65% at ninety days; earlier indicators may be internal only and do not replace disbursement measurement.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Recommending 60-day reporting as primary metric is a red line.</t>
+          <t>Red line if a team elevates a shorter window (e.g. 60-day) as the primary Board/donor metric to look better. Strong teams catch this by reading the grant, not by being told.</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1267,12 +1295,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Team names, roles, scope, request protocol agreed, online confirm by deadline.</t>
+          <t>Team names, roles, scope, A↔B evidence loop agreed, online confirm by deadline.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Charter confirmed; RACI has one accountable owner; A/B data rule stated.</t>
+          <t>Charter confirmed; RACI has one accountable owner; Estate→Demand→Plan→R/FM rule stated.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
@@ -1304,17 +1332,17 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>One precise problem sentence; MECE branches; 4+ hypotheses that imply asks for B.</t>
+          <t>One precise decision sentence in the team's own words; MECE branches they invent; 4+ hypotheses that imply asks for B.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Hypotheses map to Analysis Requests; no overlap between branches.</t>
+          <t>Hypotheses map to Analysis Requests; branches emerge from evidence; statement sharpens the engagement letter.</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Restates handbook verbatim; generic tree; no implied asks.</t>
+          <t>Copies engagement-letter wording; generic or pre-labelled tree; no implied asks.</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1406,7 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Every shared D-01 to D-12 source rated H/M/L with justification; Findings Memos rated once received.</t>
+          <t>Every shared client document (D-01, D-02, D-03, D-08, D-10, D-11, D-12) rated H/M/L with justification; Findings Memos rated once received.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -1395,17 +1423,17 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Analysis Requests (min. 3)</t>
+          <t>Data Estate Brief</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Weeks 3-5</t>
+          <t>Mon Week 3</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1415,34 +1443,34 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Each request states decision, hypothesis, useful answer shape, urgency; logged on Request Log.</t>
+          <t>Catalog of tables, grain, coverage and limits in plain language. No workbook, dictionary or field dump.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Asks are specific enough for B to answer; emerge from transcripts/hypotheses.</t>
+          <t>A can aim Demand without seeing raw data; limits are honest; catalog not a spoiler of findings.</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Fewer than three; vague 'send us the data'; field names invented from nowhere.</t>
+          <t>Raw file shared; schema dump that lets A prescribe joins; empty or late brief.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>B1 - Data quality report</t>
+          <t>Demand Brief</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Tue 11 Aug</t>
+          <t>Mon-Tue Week 3</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1452,24 +1480,24 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>DC-01 to DC-13 found or consciously checked; cleaning logged; A gets only material issues via FM.</t>
+          <t>Ranked decision needs from A1 hypotheses after reading DEB; useful answer shapes; not column shopping.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>Duplicates, coding, typo wage, DN double-entry, text funding row all addressed.</t>
+          <t>Top demands map to R-01+; each would change the recommendation if answered.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Silent cleaning; raw file shared with A; claims 100% clean data.</t>
+          <t>Vague 'send us the data'; field names invented; filed before reading Estate Brief.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Findings Memos (min. 3)</t>
+          <t>Analysis Plans</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -1479,7 +1507,7 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Weeks 3-5</t>
+          <t>From Week 3</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1489,24 +1517,24 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Plain-language answers to R-xx; definitions and caveats; curated charts only.</t>
+          <t>B-owned approach for each priority Demand / R-xx: method, definitions, risks, ETA.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Restates question; translates honestly; notes sample limitation.</t>
+          <t>Plan answers A's decision question; A acknowledges without co-editing pivots.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Pivot dump; no caveats; raw workbook attached.</t>
+          <t>No plan; plan is a field list for A to run; interim raw extracts shared.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>A2 - Interview synthesis</t>
+          <t>Analysis Requests (min. 3)</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -1516,7 +1544,7 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Wed 12 Aug</t>
+          <t>Weeks 3-5</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1526,34 +1554,34 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Thematic summary with transcript refs; contradictions flagged; questions for B listed.</t>
+          <t>Each request states decision, hypothesis, useful answer shape, urgency; linked to Demand/Plan; logged on Request Log.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Themes: transport, employer quality, metric integrity, scale vs quality.</t>
+          <t>Asks are specific enough for B to answer; emerge from Demand + transcripts/hypotheses.</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Quote dump by person; no contradictions; no citations.</t>
+          <t>Fewer than three; vague 'send us the data'; field names invented from nowhere; no Demand/Plan trail.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>A3 - Empathy and journey maps</t>
+          <t>B1 - Data quality report</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Wed 12 Aug</t>
+          <t>Tue 11 Aug</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1563,24 +1591,24 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>One archetype grounded in BN-xx; pain points with quotes or FM cites.</t>
+          <t>DC-01 to DC-14 found or consciously checked; cleaning logged; A gets only material issues via FM.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Internship stage shows transport cost and employer exploitation; links to ST-05 and EP-02.</t>
+          <t>Duplicates (via last_updated), coding, typo wage, DN double-entry, inactive mentor, text funding row addressed.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Generic persona; no quotes; outside-in design with no lived detail.</t>
+          <t>Silent cleaning; raw file shared with A; claims 100% clean data.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>B2 - Performance dashboard</t>
+          <t>Findings Memos (min. 3)</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -1590,44 +1618,44 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Fri 14 Aug</t>
+          <t>Weeks 3-5</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Placement by hub/programme/gender; flag below 65%; insight-titled charts; B working file only.</t>
+          <t>Plain-language answers to R-xx; definitions and caveats; curated charts only.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>DN and Long An flagged; formal vs broad rate shown or footnoted.</t>
+          <t>Restates question; translates honestly; states placement definition and capacity caveats.</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>Shared raw with A; DN hidden; single blended rate with no definition.</t>
+          <t>Pivot dump; no caveats; raw workbook attached.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>B3 - Analysis summary</t>
+          <t>A2 - Interview synthesis</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Wed 19 Aug</t>
+          <t>Wed 12 Aug</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1637,24 +1665,24 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Headline findings linked to Request/FM IDs; confounders named.</t>
+          <t>Thematic summary with transcript refs; contradictions flagged; questions for B listed.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Attendance correlates with placement but transport/motivation confound.</t>
+          <t>Themes: transport, employer quality, metric integrity, scale vs quality.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Claims attendance causes placement; ignores confounders.</t>
+          <t>Quote dump by person; no contradictions; no citations.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>A4 - Strategic options</t>
+          <t>A3 - Empathy and journey maps</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
@@ -1664,7 +1692,7 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Thu 20 Aug</t>
+          <t>Wed 12 Aug</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -1674,24 +1702,24 @@
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>2-3 distinct options; every number cites R-/FM-; winners/losers named.</t>
+          <t>One archetype grounded in BN-xx; pain points with quotes or FM cites.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Options differ on scale timing; change-my-mind trigger stated.</t>
+          <t>Internship stage shows transport cost and employer exploitation; links to ST-05 and EP-02.</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Three variants of 'scale more'; numbers without Request IDs.</t>
+          <t>Generic persona; no quotes; outside-in design with no lived detail.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>B4 - Evidence-check memo</t>
+          <t>B2 - Performance dashboard</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -1701,44 +1729,44 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Fri 21 Aug</t>
+          <t>Fri 14 Aug</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>PDF</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Each A option tested against Findings and D-12/D-03 feasibility.</t>
+          <t>Placement by hub/programme/gender; flag below 65%; insight-titled charts; B working file only.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Flags if aggressive growth cannot hold 65% without selection pressure.</t>
+          <t>DN and Long An flagged; formal vs broad rate shown or footnoted.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Rubber-stamps A without challenge.</t>
+          <t>Shared raw with A; DN hidden; single blended rate with no definition.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>A5 - Trade-off reflection</t>
+          <t>B3 - Analysis summary</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Wed 26 Aug</t>
+          <t>Wed 19 Aug</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -1748,34 +1776,34 @@
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Open prompts answered; who gains/loses; cost of preferred path named.</t>
+          <t>Headline findings linked to Request/FM IDs; confounders named.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>Team names the operational cost of the ethical choice, or the moral cost of the efficient choice.</t>
+          <t>Attendance correlates with placement but transport/motivation confound.</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Empty platitudes; no named cost; checklist of invented ED codes.</t>
+          <t>Claims attendance causes placement; ignores confounders.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>A6 - Validation protocol</t>
+          <t>A4 - Strategic options</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Wed 26 Aug</t>
+          <t>Thu 20 Aug</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -1785,24 +1813,24 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>6+ citations including BN/ST/DN/EP and at least two R-/FM-.</t>
+          <t>2-3 distinct options; every number cites R-/FM-; winners/losers named.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Dong Nai recommendation cites ST-05, BN-02, EP-02 and FM findings.</t>
+          <t>Options differ on scale timing; change-my-mind trigger stated.</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Validation after the fact; fewer than six citations.</t>
+          <t>Three variants of 'scale more'; numbers without Request IDs.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>B5 - Funding scenarios</t>
+          <t>B4 - Evidence-check memo</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1812,44 +1840,44 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Thu 27 Aug</t>
+          <t>Fri 21 Aug</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Hold / +30% / +80% using D-12 and D-03.</t>
+          <t>Each A option tested against Findings and D-12/D-03 feasibility.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>Aggressive scenario shows staffing gap and 65% at risk.</t>
+          <t>Flags if aggressive growth cannot hold 65% without selection pressure.</t>
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Assumes 65% holds automatically.</t>
+          <t>Rubber-stamps A without challenge.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>A7 - Revision log</t>
+          <t>A5 - Trade-off reflection</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>A</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Thu 27 Aug</t>
+          <t>Wed 26 Aug</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1859,24 +1887,24 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>At least one substantive change after a B challenge or Findings Memo.</t>
+          <t>Open prompts answered; who gains/loses; cost of preferred path named.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Example: dropped Long An expansion after FM on DN placement.</t>
+          <t>Team names the operational cost of the ethical choice, or the moral cost of the efficient choice.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Empty log or cosmetic edits only.</t>
+          <t>Empty platitudes; no named cost; checklist of invented ED codes.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Executive summary</t>
+          <t>A6 - Validation protocol</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1886,7 +1914,7 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Fri 28 Aug</t>
+          <t>Wed 26 Aug</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -1896,61 +1924,61 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>One-sentence key message; recommendation; 90-day roadmap; honest limitations.</t>
+          <t>6+ citations including BN/ST/DN/EP and at least two R-/FM-.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>Board-ready; cites strongest evidence including Request IDs.</t>
+          <t>Dong Nai recommendation cites ST-05, BN-02, EP-02 and FM findings.</t>
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>Buries recommendation; no limitations.</t>
+          <t>Validation after the fact; fewer than six citations.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Final report</t>
+          <t>B5 - Funding scenarios</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Fri 11 Sep</t>
+          <t>Thu 27 Aug</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>PDF</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>15-25 pages; request protocol described; every claim sourced.</t>
+          <t>Hold / +30% / +80% using D-12, D-03 and hub_capacity_jan2026.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Integrates A narrative and B findings; trade-offs and risks included.</t>
+          <t>Aggressive scenario shows staffing/mentor gap and 65% at risk; ties choice to mission + Board ambition.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>A and B contradict; unsourced numbers; raw data pasted.</t>
+          <t>Assumes 65% holds automatically; ignores staff/mentor/finance capacity.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Board presentation</t>
+          <t>A7 - Revision log</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
@@ -1960,64 +1988,249 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Thu 10 Sep</t>
+          <t>Thu 27 Aug</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>PowerPoint</t>
+          <t>PDF</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Answer-first titles; Dong Nai and formal rate not hidden; cost of path named.</t>
+          <t>At least one substantive change after a B challenge or Findings Memo.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>Opens with decision needed; ends with specific Board asks.</t>
+          <t>Example: dropped Long An expansion after FM on DN placement.</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>Data dump; no clear ask; A cites 'the dataset' without FM IDs.</t>
+          <t>Empty log or cosmetic edits only.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>Executive summary</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Fri 28 Aug</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>One-sentence key message; recommendation; 90-day roadmap; honest limitations.</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Board-ready; cites strongest evidence including Request IDs.</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>Buries recommendation; no limitations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Final report</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Fri 11 Sep</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>15-25 pages; A↔B evidence loop described; every claim sourced.</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Integrates A narrative and B findings; trade-offs and risks included.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>A and B contradict; unsourced numbers; raw data pasted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Board presentation</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Thu 10 Sep</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>PowerPoint</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Answer-first titles; Dong Nai and formal rate not hidden; cost of path named.</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Opens with decision needed; ends with specific Board asks.</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Data dump; no clear ask; A cites 'the dataset' without FM IDs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
           <t>Handoff checklist</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Wed 2 Sep</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>PDF</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>Both sections online-confirmed; Request Log shows min. three completed pairs.</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Genuine exchange evidenced; Engagement Lead confirms in good faith.</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>One dump at the end; raw file shared; unchecked.</t>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>Copy 4_Shared_Toolkit/Templates/Cross_Workflow_Handoff_Checklist.docx to team Drive. Section A (A reviews B), Section B (B reviews A), Section C (Engagement Lead). Online ticks only: [x] + typed name + YYYY-MM-DD + channel. Export Team_All_Handoff_vN.pdf; Request Log shows min. three completed R/FM pairs. See Guideline Section 8.</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>All three sections confirmed; Drive links to A_B_Exchange/ and Handoff PDF present; genuine exchange (not a last-minute dump).</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>Missing PDF; wet-signature / print culture; unchecked boxes; fewer than three R/FM pairs; raw file shared with A.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Peer evaluation</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Mon 14 Sep</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Confidential peer ratings for each teammate; submitted individually via portal.</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Honest differentiation; comments specific to contribution.</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>Identical scores for everyone; blank comments; late or missing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Reflection journal</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Tue 15 Sep</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>PDF</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Personal learning reflection on the engagement and cross-workflow practice.</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Names a concrete skill and a cost of the team's recommendation.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>Generic essay; no link to the case evidence or teamwork.</t>
         </is>
       </c>
     </row>

</xml_diff>